<commit_message>
Tufts capacity retirements and guaranteed dispatch data corrections
</commit_message>
<xml_diff>
--- a/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
+++ b/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BGDPbES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AB2B1E-2998-B643-B477-BFCD12DF6B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294C88A3-4B51-9944-B44D-BBFD2A19C196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="354">
   <si>
     <t>Notes:</t>
   </si>
@@ -1092,13 +1092,19 @@
   </si>
   <si>
     <t>Bid Capacity Factor x Hours per Year[municipal solid waste es,newly built] : MostRecentRun</t>
+  </si>
+  <si>
+    <t>BPS</t>
+  </si>
+  <si>
+    <t>https://esdm.go.id/assets/media/content/content-handbook-of-energy-and-economic-statistics-of-indonesia-2023.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1121,6 +1127,14 @@
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1139,10 +1153,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1159,8 +1174,10 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1463,7 +1480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1500,53 +1517,66 @@
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="1" t="s">
-        <v>0</v>
+      <c r="B9" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" t="s">
+      <c r="B10" s="8" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
         <v>282</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{AE7F4E09-2A8B-E04F-9419-569707F06952}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -15193,128 +15223,97 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <f>'2020 Calculations'!B2</f>
-        <v>0.4676053280482092</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>'2020 Calculations'!C2</f>
-        <v>0.38725783384127582</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>'2020 Calculations'!D2</f>
-        <v>0.36299246943702695</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <f>'2020 Calculations'!E2</f>
-        <v>0.3235427622169037</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <f>'2020 Calculations'!F2</f>
-        <v>0.29232541068905493</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <f>'2020 Calculations'!G2</f>
-        <v>0.27314691896863608</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <f>'2020 Calculations'!H2</f>
-        <v>0.25748079133253876</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <f>'2020 Calculations'!I2</f>
-        <v>0.24465157886158045</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <f>'2020 Calculations'!J2</f>
-        <v>0.23436231549722417</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <f>'2020 Calculations'!K2</f>
-        <v>0.22580521187310026</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <f>'2020 Calculations'!L2</f>
-        <v>0.21860014601771138</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <f>'2020 Calculations'!M2</f>
-        <v>0.22690057069799094</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <f>'2020 Calculations'!N2</f>
-        <v>0.23520099537827049</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <f>'2020 Calculations'!O2</f>
-        <v>0.24350142005854736</v>
+        <v>0</v>
       </c>
       <c r="U2">
-        <f>'2020 Calculations'!P2</f>
-        <v>0.25180184473882694</v>
+        <v>0</v>
       </c>
       <c r="V2">
-        <f>'2020 Calculations'!Q2</f>
-        <v>0.26010226941910647</v>
+        <v>0</v>
       </c>
       <c r="W2">
-        <f>'2020 Calculations'!R2</f>
-        <v>0.26840269409938605</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <f>'2020 Calculations'!S2</f>
-        <v>0.27670311877966286</v>
+        <v>0</v>
       </c>
       <c r="Y2">
-        <f>'2020 Calculations'!T2</f>
-        <v>0.28500354345994244</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <f>'2020 Calculations'!U2</f>
-        <v>0.29330396814022197</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <f>'2020 Calculations'!V2</f>
-        <v>0.30160439282049883</v>
+        <v>0</v>
       </c>
       <c r="AB2">
-        <f>'2020 Calculations'!W2</f>
-        <v>0.30990481750077842</v>
+        <v>0</v>
       </c>
       <c r="AC2">
-        <f>'2020 Calculations'!X2</f>
-        <v>0.318205242181058</v>
+        <v>0</v>
       </c>
       <c r="AD2">
-        <f>'2020 Calculations'!Y2</f>
-        <v>0.32650566686133481</v>
+        <v>0</v>
       </c>
       <c r="AE2">
-        <f>'2020 Calculations'!Z2</f>
-        <v>0.33480609154161439</v>
+        <v>0</v>
       </c>
       <c r="AF2">
-        <f>'2020 Calculations'!AA2</f>
-        <v>0.34310651622189392</v>
+        <v>0</v>
       </c>
       <c r="AG2">
-        <f>'2020 Calculations'!AB2</f>
-        <v>0.3514069409021735</v>
+        <v>0</v>
       </c>
       <c r="AH2">
-        <f>'2020 Calculations'!AC2</f>
-        <v>0.35970736558245037</v>
+        <v>0</v>
       </c>
       <c r="AI2">
-        <f>'2020 Calculations'!AD2</f>
-        <v>0.36800779026272995</v>
+        <v>0</v>
       </c>
       <c r="AJ2">
-        <f>'2020 Calculations'!AE2</f>
-        <v>0.37630821494300948</v>
+        <v>0</v>
       </c>
       <c r="AK2">
-        <f>'2020 Calculations'!AF2</f>
-        <v>0.38460863962328634</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:37">
@@ -15346,115 +15345,87 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:R3" si="0">$B3</f>
         <v>0</v>
       </c>
       <c r="K3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="N3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R3">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S3">
-        <f t="shared" ref="J3:AK9" si="1">$B3</f>
         <v>0</v>
       </c>
       <c r="T3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AK3">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -15487,115 +15458,87 @@
         <v>0</v>
       </c>
       <c r="J4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AK4">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -15628,115 +15571,87 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AK5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -15769,115 +15684,87 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AK6">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -15910,115 +15797,87 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AK7">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16051,115 +15910,87 @@
         <v>0</v>
       </c>
       <c r="J8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AK8">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16192,115 +16023,87 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AA9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AC9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AE9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AF9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AG9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AH9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AI9">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AJ9">
-        <f t="shared" ref="G9:AK14" si="2">$B9</f>
         <v>0</v>
       </c>
       <c r="AK9">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -16333,115 +16136,87 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="W10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="X10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Y10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AA10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AB10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AD10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AG10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AH10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AJ10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK10">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -16474,115 +16249,87 @@
         <v>0</v>
       </c>
       <c r="J11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="W11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="X11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Y11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AA11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AB11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AD11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AG11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AH11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AJ11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK11">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -16606,127 +16353,96 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="H12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="W12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="X12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Y12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AA12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AB12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AD12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AG12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AH12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AJ12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK12">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -16750,128 +16466,97 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <f>'2020 Calculations'!B3</f>
-        <v>0.40441541885250526</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <f>'2020 Calculations'!C3</f>
-        <v>0.38725783384127582</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <f>'2020 Calculations'!D3</f>
-        <v>0.36299246943702695</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <f>'2020 Calculations'!E3</f>
-        <v>0.3235427622169037</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <f>'2020 Calculations'!F3</f>
-        <v>0.29232541068905493</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <f>'2020 Calculations'!G3</f>
-        <v>0.27314691896863608</v>
+        <v>0</v>
       </c>
       <c r="M13">
-        <f>'2020 Calculations'!H3</f>
-        <v>0.25748079133253876</v>
+        <v>0</v>
       </c>
       <c r="N13">
-        <f>'2020 Calculations'!I3</f>
-        <v>0.24465157886158045</v>
+        <v>0</v>
       </c>
       <c r="O13">
-        <f>'2020 Calculations'!J3</f>
-        <v>0.23436231549722417</v>
+        <v>0</v>
       </c>
       <c r="P13">
-        <f>'2020 Calculations'!K3</f>
-        <v>0.22580521187310026</v>
+        <v>0</v>
       </c>
       <c r="Q13">
-        <f>'2020 Calculations'!L3</f>
-        <v>0.21860014601771138</v>
+        <v>0</v>
       </c>
       <c r="R13">
-        <f>'2020 Calculations'!M3</f>
-        <v>0.22690057069799094</v>
+        <v>0</v>
       </c>
       <c r="S13">
-        <f>'2020 Calculations'!N3</f>
-        <v>0.23520099537827049</v>
+        <v>0</v>
       </c>
       <c r="T13">
-        <f>'2020 Calculations'!O3</f>
-        <v>0.24350142005854736</v>
+        <v>0</v>
       </c>
       <c r="U13">
-        <f>'2020 Calculations'!P3</f>
-        <v>0.25180184473882694</v>
+        <v>0</v>
       </c>
       <c r="V13">
-        <f>'2020 Calculations'!Q3</f>
-        <v>0.26010226941910647</v>
+        <v>0</v>
       </c>
       <c r="W13">
-        <f>'2020 Calculations'!R3</f>
-        <v>0.26840269409938605</v>
+        <v>0</v>
       </c>
       <c r="X13">
-        <f>'2020 Calculations'!S3</f>
-        <v>0.27670311877966286</v>
+        <v>0</v>
       </c>
       <c r="Y13">
-        <f>'2020 Calculations'!T3</f>
-        <v>0.28500354345994244</v>
+        <v>0</v>
       </c>
       <c r="Z13">
-        <f>'2020 Calculations'!U3</f>
-        <v>0.29330396814022197</v>
+        <v>0</v>
       </c>
       <c r="AA13">
-        <f>'2020 Calculations'!V3</f>
-        <v>0.30160439282049883</v>
+        <v>0</v>
       </c>
       <c r="AB13">
-        <f>'2020 Calculations'!W3</f>
-        <v>0.30990481750077842</v>
+        <v>0</v>
       </c>
       <c r="AC13">
-        <f>'2020 Calculations'!X3</f>
-        <v>0.318205242181058</v>
+        <v>0</v>
       </c>
       <c r="AD13">
-        <f>'2020 Calculations'!Y3</f>
-        <v>0.32650566686133481</v>
+        <v>0</v>
       </c>
       <c r="AE13">
-        <f>'2020 Calculations'!Z3</f>
-        <v>0.33480609154161439</v>
+        <v>0</v>
       </c>
       <c r="AF13">
-        <f>'2020 Calculations'!AA3</f>
-        <v>0.34310651622189392</v>
+        <v>0</v>
       </c>
       <c r="AG13">
-        <f>'2020 Calculations'!AB3</f>
-        <v>0.3514069409021735</v>
+        <v>0</v>
       </c>
       <c r="AH13">
-        <f>'2020 Calculations'!AC3</f>
-        <v>0.35970736558245037</v>
+        <v>0</v>
       </c>
       <c r="AI13">
-        <f>'2020 Calculations'!AD3</f>
-        <v>0.36800779026272995</v>
+        <v>0</v>
       </c>
       <c r="AJ13">
-        <f>'2020 Calculations'!AE3</f>
-        <v>0.37630821494300948</v>
+        <v>0</v>
       </c>
       <c r="AK13">
-        <f>'2020 Calculations'!AF3</f>
-        <v>0.38460863962328634</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -16906,111 +16591,84 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="W14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="X14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Y14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Z14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AA14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AB14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AD14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AG14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AH14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AJ14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK14">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -17260,135 +16918,101 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <f t="shared" ref="G17:AK17" si="3">F17</f>
         <v>0</v>
       </c>
       <c r="H17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="S17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="V17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="W17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="X17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Y17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Z17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AB17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AC17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AD17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AE17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AG17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AH17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AI17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AJ17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AK17">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <ignoredErrors>
-    <ignoredError sqref="K13:Q13 R13:AK13" formula="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>